<commit_message>
Page 404 : liens de la rubrique OKILYS Suite passes en chemin absolu
Les entrees suite.html, ctms.html et etmf.html du menu de la page 404 etaient en chemin relatif
alors que tous les autres liens de cette page sont absolus. Une erreur survenant dans un
sous-dossier (par exemple /en/adresse-inexistante) resolvait ces liens au mauvais endroit.
Defaut trouve en jouant ST-PAGE-06 au navigateur le 19/09.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_notes/validation/resultats-tests-site-web-20260919a.xlsx
+++ b/_notes/validation/resultats-tests-site-web-20260919a.xlsx
@@ -477,7 +477,7 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Un seul onglet, 1 defauts (echecs) + 40 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur la colonne 'Action souhaitee' pour ne montrer que les lignes ou vous n'avez PAS encore demande de correction. Pour revoir tout l'historique (y compris ce que vous avez deja decide, ou les points corriges/plus detectes), enlevez le filtre de la colonne 'Action souhaitee'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
+          <t>Un seul onglet, 1 defauts (echecs) + 23 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
         </is>
       </c>
     </row>
-    <row r="5" hidden="1">
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>PT-DNS-01</t>
@@ -581,7 +581,7 @@
       </c>
       <c r="J5" s="4" t="n"/>
     </row>
-    <row r="6" hidden="1">
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>IT-FORM-02</t>
@@ -629,7 +629,7 @@
       </c>
       <c r="J6" s="4" t="n"/>
     </row>
-    <row r="7" hidden="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>IT-FORM-03</t>
@@ -681,10 +681,10 @@
         </is>
       </c>
     </row>
-    <row r="8" hidden="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PT-CLICK-01</t>
+          <t>PT-DNS-02</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -699,22 +699,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Clickjacking</t>
+          <t>Zone hygiene</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Test de « mise en cadre » du site (clickjacking) : à confirmer dans un navigateur ; GitHub Pages ne permet pas d'ajouter l'en-tête de protection habituel.</t>
+          <t>Réglages du nom de domaine à contrôler chez le bureau d'enregistrement (registrar) : verrouillage du domaine, signature DNSSEC, enregistrement CAA. Nécessite l'accès au compte du domaine.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer en navigateur.</t>
+          <t>Aucun défaut détecté : à confirmer côté registrar.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Clickjacking (framing) : à confirmer en navigateur ; en-têtes X-Frame-Options/CSP non modifiables sur GitHub Pages.</t>
+          <t>DNS/registrar : verrou de transfert, DNSSEC, enregistrement CAA (optionnel). Nécessite l'accès au registrar.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -733,10 +733,10 @@
         </is>
       </c>
     </row>
-    <row r="9" hidden="1">
+    <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PT-DNS-02</t>
+          <t>PT-FORM-01</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -751,22 +751,22 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Zone hygiene</t>
+          <t>Form abuse</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Réglages du nom de domaine à contrôler chez le bureau d'enregistrement (registrar) : verrouillage du domaine, signature DNSSEC, enregistrement CAA. Nécessite l'accès au compte du domaine.</t>
+          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer côté registrar.</t>
+          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>DNS/registrar : verrou de transfert, DNSSEC, enregistrement CAA (optionnel). Nécessite l'accès au registrar.</t>
+          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -785,10 +785,10 @@
         </is>
       </c>
     </row>
-    <row r="10" hidden="1">
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-01</t>
+          <t>PT-FORM-02</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Form abuse</t>
+          <t>Rate and quota</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -837,10 +837,10 @@
         </is>
       </c>
     </row>
-    <row r="11" hidden="1">
+    <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-02</t>
+          <t>PT-FORM-03</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Rate and quota</t>
+          <t>Privacy of submissions</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -889,10 +889,10 @@
         </is>
       </c>
     </row>
-    <row r="12" hidden="1">
+    <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-03</t>
+          <t>PT-FORM-04</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Privacy of submissions</t>
+          <t>Bot / spam traps and key scraping</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -941,10 +941,10 @@
         </is>
       </c>
     </row>
-    <row r="13" hidden="1">
+    <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-04</t>
+          <t>PT-INPUT-01</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Bot / spam traps and key scraping</t>
+          <t>Input validation (WSTG-INPV)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -993,10 +993,10 @@
         </is>
       </c>
     </row>
-    <row r="14" hidden="1">
+    <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>PT-INPUT-01</t>
+          <t>PT-SUPPLY-01</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1011,22 +1011,22 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Input validation (WSTG-INPV)</t>
+          <t>Supply chain</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1045,10 +1045,10 @@
         </is>
       </c>
     </row>
-    <row r="15" hidden="1">
+    <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PT-PRIV-01</t>
+          <t>PT-TLS-02</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1063,22 +1063,22 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Privacy</t>
+          <t>HSTS</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Vérification « zéro cookie / zéro traqueur » en conditions réelles : à confirmer dans un navigateur en naviguant sur le site en ligne.</t>
+          <t>Note complète du chiffrement HTTPS (versions, algorithmes) : se mesure avec un outil externe (SSL Labs) sur le domaine en ligne, pas dans ce contrôle automatique.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer en navigation réelle.</t>
+          <t>Aucun défaut détecté : à mesurer sur le domaine en ligne.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Absence de cookies / traqueurs en conditions réelles : à confirmer via les outils du navigateur sur le site déployé.</t>
+          <t>Grade TLS complet (protocoles, ciphers) : nécessite testssl.sh / SSL Labs sur le domaine public.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1097,10 +1097,10 @@
         </is>
       </c>
     </row>
-    <row r="16" hidden="1">
+    <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-01</t>
+          <t>ST-CONTACT-02</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1110,32 +1110,32 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Supply chain</t>
+          <t>same from EN</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Toi (accès ou accord requis)</t>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1149,10 +1149,10 @@
         </is>
       </c>
     </row>
-    <row r="17" hidden="1">
+    <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-02</t>
+          <t>ST-CONTACT-03</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1162,32 +1162,32 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Publication integrity</t>
+          <t>offline (devtools)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Toi (accès ou accord requis)</t>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
@@ -1201,10 +1201,10 @@
         </is>
       </c>
     </row>
-    <row r="18" hidden="1">
+    <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PT-TLS-02</t>
+          <t>ST-CONTACT-04</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1214,32 +1214,32 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>HSTS</t>
+          <t>e-mail / phone links</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Note complète du chiffrement HTTPS (versions, algorithmes) : se mesure avec un outil externe (SSL Labs) sur le domaine en ligne, pas dans ce contrôle automatique.</t>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à mesurer sur le domaine en ligne.</t>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Grade TLS complet (protocoles, ciphers) : nécessite testssl.sh / SSL Labs sur le domaine public.</t>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Testeur / navigateur</t>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1253,10 +1253,10 @@
         </is>
       </c>
     </row>
-    <row r="19" hidden="1">
+    <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-02</t>
+          <t>ST-MOB-03</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>keyboard only</t>
+          <t>carousel</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1305,10 +1305,10 @@
         </is>
       </c>
     </row>
-    <row r="20" hidden="1">
+    <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-03</t>
+          <t>ST-MOB-04</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1323,7 +1323,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>screen reader (NVDA) on the home</t>
+          <t>contact</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1357,10 +1357,10 @@
         </is>
       </c>
     </row>
-    <row r="21" hidden="1">
+    <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-04</t>
+          <t>ST-NAV-05</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>contrast and zoom</t>
+          <t>back / forward</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1409,10 +1409,10 @@
         </is>
       </c>
     </row>
-    <row r="22" hidden="1">
+    <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-05</t>
+          <t>ST-PAGE-01</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>motion</t>
+          <t>5 product pages</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1461,10 +1461,10 @@
         </is>
       </c>
     </row>
-    <row r="23" hidden="1">
+    <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-02</t>
+          <t>ST-PAGE-02</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>same from EN</t>
+          <t>7 step pages</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -1513,10 +1513,10 @@
         </is>
       </c>
     </row>
-    <row r="24" hidden="1">
+    <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-03</t>
+          <t>ST-PAGE-03</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>offline (devtools)</t>
+          <t>About page</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1565,10 +1565,10 @@
         </is>
       </c>
     </row>
-    <row r="25" hidden="1">
+    <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-04</t>
+          <t>ST-PAGE-04</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>e-mail / phone links</t>
+          <t>Réalisations and Actualités</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
@@ -1617,10 +1617,10 @@
         </is>
       </c>
     </row>
-    <row r="26" hidden="1">
+    <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-01</t>
+          <t>ST-PAGE-06</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>hero and figures band</t>
+          <t>Legal and 404</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1669,10 +1669,10 @@
         </is>
       </c>
     </row>
-    <row r="27" hidden="1">
+    <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-03</t>
+          <t>ST-PERF-02</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>À propos + HOME tiles</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -1721,10 +1721,10 @@
         </is>
       </c>
     </row>
-    <row r="28" hidden="1">
+    <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-04</t>
+          <t>ST-PERF-03</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Produits de santé and Expertises</t>
+          <t>cache behaviour after a publication</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1776,44 +1776,32 @@
     <row r="29" hidden="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-05</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>IT-NAV-03</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intégration</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Secteurs, OKILYS Suite panel, Contact</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
       <c r="I29" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -1821,51 +1809,39 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Joue ce test toi-même.</t>
+          <t>Harmonise, garde le nom le plus court</t>
         </is>
       </c>
     </row>
     <row r="30" hidden="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-03</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>PT-CLICK-01</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>carousel</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -1880,96 +1856,68 @@
     <row r="31" hidden="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-04</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>PT-HDR-01</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>contact</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
+      <c r="J31" s="4" t="n"/>
     </row>
     <row r="32" hidden="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-05</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>PT-PRIV-01</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>tablet 768 px</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -1984,44 +1932,32 @@
     <row r="33" hidden="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>ST-NAV-03</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>PT-SUPPLY-02</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>scrollspy</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
       <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2036,12 +1972,12 @@
     <row r="34" hidden="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ST-NAV-05</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-A11Y-02</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2051,29 +1987,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>back / forward</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2088,12 +2012,12 @@
     <row r="35" hidden="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-01</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-A11Y-03</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2103,29 +2027,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>5 product pages</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
       <c r="I35" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2140,12 +2052,12 @@
     <row r="36" hidden="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-02</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-A11Y-04</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2155,29 +2067,17 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>7 step pages</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
       <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2192,12 +2092,12 @@
     <row r="37" hidden="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-03</t>
-        </is>
-      </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-A11Y-05</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2207,29 +2107,17 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>About page</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
       <c r="I37" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2244,12 +2132,12 @@
     <row r="38" hidden="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-04</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-HOME-01</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2259,29 +2147,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Réalisations and Actualités</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2296,12 +2172,12 @@
     <row r="39" hidden="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ST-PAGE-06</t>
-        </is>
-      </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-HOME-03</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2311,29 +2187,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Legal and 404</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2348,12 +2212,12 @@
     <row r="40" hidden="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ST-PERF-02</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-HOME-04</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2363,29 +2227,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>fonts</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2400,12 +2252,12 @@
     <row r="41" hidden="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ST-PERF-03</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-HOME-05</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2415,29 +2267,17 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>cache behaviour after a publication</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
       <c r="I41" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2452,12 +2292,12 @@
     <row r="42" hidden="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-02</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-MOB-05</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2467,29 +2307,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Google Rich Results test on home, About, a product page, `ctms`</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr"/>
       <c r="I42" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2504,12 +2332,12 @@
     <row r="43" hidden="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-03</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-NAV-03</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2519,29 +2347,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Search Console and Bing Webmaster</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
       <c r="I43" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2556,12 +2372,12 @@
     <row r="44" hidden="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-04</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-SEO-02</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2571,29 +2387,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>hreflang validator (e.g. Merkle / Sistrix) on 6 pages</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
       <c r="I44" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2608,12 +2412,12 @@
     <row r="45" hidden="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>ST-SEO-05</t>
-        </is>
-      </c>
-      <c r="B45" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>ST-SEO-03</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2623,29 +2427,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>snippet preview</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -2660,7 +2452,7 @@
     <row r="46" hidden="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>IT-NAV-03</t>
+          <t>ST-SEO-04</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
@@ -2670,7 +2462,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -2693,14 +2485,14 @@
       </c>
       <c r="J46" s="4" t="inlineStr">
         <is>
-          <t>Harmonise, garde le nom le plus court</t>
+          <t>Joue ce test toi-même.</t>
         </is>
       </c>
     </row>
     <row r="47" hidden="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>PT-HDR-01</t>
+          <t>ST-SEO-05</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
@@ -2710,7 +2502,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -2731,7 +2523,11 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J47" s="4" t="n"/>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
     </row>
     <row r="48" hidden="1">
       <c r="A48" s="2" t="inlineStr">
@@ -2847,8 +2643,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:J50">
-    <filterColumn colId="8" hiddenButton="0" showButton="1">
-      <filters blank="1"/>
+    <filterColumn colId="1" hiddenButton="0" showButton="1">
+      <filters blank="0">
+        <filter val="Bloqué"/>
+        <filter val="Mineur"/>
+      </filters>
     </filterColumn>
   </autoFilter>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Specification de tests du site : corrections issues des tests joues le 19/09
- ST-PAGE-03 : chiffres reels verifies au navigateur — 14 logos dans le mur, dont 13 cliquables en nouvel onglet securise et un seul (Azeolys) sans lien. La specification annoncait 11 logos.
- ST-CONTACT-04, ST-MOB-04, UT-JS-01 : la partie telephone est marquee SANS OBJET, aucun numero n etant publie sur le site. Volontairement marquee sans objet plutot que supprimee, la decision de publier ou non un numero appartenant a Lydie.
- Paragraphe 9 : trois points ouverts ajoutes (logo Azeolys sans lien, absence de numero de telephone, enregistrement CAA absent)

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_notes/validation/resultats-tests-site-web-20260919a.xlsx
+++ b/_notes/validation/resultats-tests-site-web-20260919a.xlsx
@@ -470,14 +470,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OKILYS site web (www.okilys.com) - Cas a revoir (version 20260919a) - execute le 2026-09-19T21:27:35.904524</t>
+          <t>OKILYS site web (www.okilys.com) - Cas a revoir (version 20260919a) - execute le 2026-09-19T21:41:43.252506</t>
         </is>
       </c>
     </row>
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Un seul onglet, 1 defauts (echecs) + 23 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
+          <t>Un seul onglet, 1 defauts (echecs) + 11 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
         </is>
       </c>
     </row>
@@ -1048,7 +1048,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PT-TLS-02</t>
+          <t>ST-CONTACT-02</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1058,32 +1058,32 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>HSTS</t>
+          <t>same from EN</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Note complète du chiffrement HTTPS (versions, algorithmes) : se mesure avec un outil externe (SSL Labs) sur le domaine en ligne, pas dans ce contrôle automatique.</t>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à mesurer sur le domaine en ligne.</t>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Grade TLS complet (protocoles, ciphers) : nécessite testssl.sh / SSL Labs sur le domaine public.</t>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Testeur / navigateur</t>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
@@ -1100,7 +1100,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-02</t>
+          <t>ST-PERF-03</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1115,7 +1115,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>same from EN</t>
+          <t>cache behaviour after a publication</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1149,587 +1149,451 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>IT-NAV-03</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intégration</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>Harmonise, garde le nom le plus court</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" hidden="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>PT-CLICK-01</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intrusion</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" hidden="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>PT-HDR-01</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intrusion</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="n"/>
+    </row>
+    <row r="20" hidden="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>PT-PRIV-01</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intrusion</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" hidden="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>PT-SUPPLY-02</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intrusion</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" hidden="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>PT-TLS-02</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intrusion</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" hidden="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ST-A11Y-02</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" hidden="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ST-A11Y-03</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" hidden="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ST-A11Y-04</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" hidden="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ST-A11Y-05</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" hidden="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>ST-CONTACT-03</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>offline (devtools)</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" hidden="1">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>ST-CONTACT-04</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>e-mail / phone links</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>ST-MOB-03</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>carousel</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>ST-MOB-04</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>contact</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>ST-NAV-05</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>back / forward</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>ST-PAGE-01</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>5 product pages</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>ST-PAGE-02</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>7 step pages</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>ST-PAGE-03</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>About page</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>ST-PAGE-04</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Réalisations and Actualités</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>ST-PAGE-06</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Legal and 404</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>ST-PERF-02</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>fonts</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>ST-PERF-03</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1739,29 +1603,17 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>cache behaviour after a publication</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -1776,7 +1628,7 @@
     <row r="29" hidden="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>IT-NAV-03</t>
+          <t>ST-HOME-01</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
@@ -1786,7 +1638,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1809,14 +1661,14 @@
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>Harmonise, garde le nom le plus court</t>
+          <t>Joue ce test toi-même.</t>
         </is>
       </c>
     </row>
     <row r="30" hidden="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>PT-CLICK-01</t>
+          <t>ST-HOME-03</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
@@ -1826,7 +1678,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1856,7 +1708,7 @@
     <row r="31" hidden="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>PT-HDR-01</t>
+          <t>ST-HOME-04</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -1866,7 +1718,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1887,12 +1739,16 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J31" s="4" t="n"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
     </row>
     <row r="32" hidden="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>PT-PRIV-01</t>
+          <t>ST-HOME-05</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
@@ -1902,7 +1758,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1932,7 +1788,7 @@
     <row r="33" hidden="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-02</t>
+          <t>ST-MOB-03</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
@@ -1942,7 +1798,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1972,7 +1828,7 @@
     <row r="34" hidden="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-02</t>
+          <t>ST-MOB-04</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -2012,7 +1868,7 @@
     <row r="35" hidden="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-03</t>
+          <t>ST-MOB-05</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -2052,7 +1908,7 @@
     <row r="36" hidden="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-04</t>
+          <t>ST-NAV-03</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -2092,7 +1948,7 @@
     <row r="37" hidden="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-05</t>
+          <t>ST-NAV-05</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
@@ -2132,7 +1988,7 @@
     <row r="38" hidden="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-01</t>
+          <t>ST-PAGE-01</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
@@ -2172,7 +2028,7 @@
     <row r="39" hidden="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-03</t>
+          <t>ST-PAGE-02</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
@@ -2212,7 +2068,7 @@
     <row r="40" hidden="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-04</t>
+          <t>ST-PAGE-03</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
@@ -2252,7 +2108,7 @@
     <row r="41" hidden="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>ST-HOME-05</t>
+          <t>ST-PAGE-04</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
@@ -2292,7 +2148,7 @@
     <row r="42" hidden="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>ST-MOB-05</t>
+          <t>ST-PAGE-06</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
@@ -2332,7 +2188,7 @@
     <row r="43" hidden="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>ST-NAV-03</t>
+          <t>ST-PERF-02</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Specification v1.6 : deux decisions de Lydie actees
- Aucun numero de telephone ne sera publie sur le site : les exigences tel: et data-tel sont
  retirees de ST-CONTACT-04, ST-MOB-04 et UT-JS-01 (l assistant dormant reste dans script.js)
- Le logo Azeolys reste volontairement sans lien : 13 logos cliquables sur 14 est l etat attendu,
  ce n est pas un defaut
- Les deux points ouverts correspondants sont retires du paragraphe 9
- Resultats des envois reels du 19/09 consignes dans l en-tete, dont l echec confirme de PT-FORM-01

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_notes/validation/resultats-tests-site-web-20260919a.xlsx
+++ b/_notes/validation/resultats-tests-site-web-20260919a.xlsx
@@ -477,7 +477,7 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Un seul onglet, 1 defauts (echecs) + 11 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
+          <t>Un seul onglet, 2 defauts (echecs) + 6 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
         </is>
       </c>
     </row>
@@ -584,42 +584,42 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>IT-FORM-02</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>PT-FORM-01</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Mineur</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>real submission FR</t>
+          <t>Formulaire de contact du site (relais Web3Forms) - pages accueil / contact</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>La cle publique du formulaire n'est pas limitee a okilys.com : quelqu'un qui la recupere (elle est lisible par le navigateur) peut envoyer des messages dans la boite de contact OKILYS depuis n'importe quel autre site. Aucune donnee du site n'est exposee et rien n'est pirate ; le seul risque est de recevoir du courrier indesirable (spam) dans la boite de contact.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Reception possible de spam dans la boite de contact OKILYS. Aucune fuite ni exposition de donnees.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>Restriction de domaine (« Allowed domains ») non activee sur la cle publique Web3Forms : une requete POST emise depuis une origine tierce (testee depuis http://localhost:8090) est acceptee (HTTP 200, message delivre). L'obfuscation de la cle ralentit les robots simples mais ne protege pas de l'execution du JavaScript de la page.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Toi (accès ou accord requis)</t>
+          <t>Tableau de bord Web3Forms &gt; reglage « Allowed domains » (compte OKILYS) - action de Lydie</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -627,12 +627,16 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J6" s="4" t="n"/>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>IT-FORM-03</t>
+          <t>PT-DNS-02</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -642,27 +646,27 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>real submission EN</t>
+          <t>Zone hygiene</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Ce test n'a pas pu être joué automatiquement : il demande une action manuelle ou un accès externe. À exécuter par le testeur.</t>
+          <t>Réglages du nom de domaine à contrôler chez le bureau d'enregistrement (registrar) : verrouillage du domaine, signature DNSSEC, enregistrement CAA. Nécessite l'accès au compte du domaine.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : reste à exécuter.</t>
+          <t>Aucun défaut détecté : à confirmer côté registrar.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Cas non automatisable dans le contrôle actuel (action manuelle ou accès externe requis).</t>
+          <t>DNS/registrar : verrou de transfert, DNSSEC, enregistrement CAA (optionnel). Nécessite l'accès au registrar.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -684,7 +688,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PT-DNS-02</t>
+          <t>PT-FORM-03</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -699,22 +703,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Zone hygiene</t>
+          <t>Privacy of submissions</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Réglages du nom de domaine à contrôler chez le bureau d'enregistrement (registrar) : verrouillage du domaine, signature DNSSEC, enregistrement CAA. Nécessite l'accès au compte du domaine.</t>
+          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à confirmer côté registrar.</t>
+          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>DNS/registrar : verrou de transfert, DNSSEC, enregistrement CAA (optionnel). Nécessite l'accès au registrar.</t>
+          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -736,7 +740,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-01</t>
+          <t>PT-FORM-04</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -751,7 +755,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Form abuse</t>
+          <t>Bot / spam traps and key scraping</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -788,7 +792,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-02</t>
+          <t>PT-SUPPLY-01</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -803,22 +807,22 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Rate and quota</t>
+          <t>Supply chain</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -840,7 +844,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-03</t>
+          <t>ST-CONTACT-02</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -850,32 +854,32 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Privacy of submissions</t>
+          <t>same from EN</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Toi (accès ou accord requis)</t>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
@@ -892,7 +896,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-04</t>
+          <t>ST-PERF-03</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -902,242 +906,190 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>Test système (navigateur)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>cache behaviour after a publication</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" hidden="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>IT-FORM-02</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intégration</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="n"/>
+    </row>
+    <row r="14" hidden="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>IT-FORM-03</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intégration</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" hidden="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>IT-NAV-03</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Test d'intégration</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>(déjà traité lors d'un test précédent)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Corriger</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>Harmonise, garde le nom le plus court</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>PT-CLICK-01</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>Test d'intrusion</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Bot / spam traps and key scraping</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Toi (accès ou accord requis)</t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>PT-INPUT-01</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Test d'intrusion</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Input validation (WSTG-INPV)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Toi (accès ou accord requis)</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>PT-SUPPLY-01</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Test d'intrusion</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Supply chain</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Toi (accès ou accord requis)</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>ST-CONTACT-02</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>same from EN</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>Corriger</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>ST-PERF-03</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Test système (navigateur)</t>
-        </is>
-      </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>cache behaviour after a publication</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -1152,7 +1104,7 @@
     <row r="17" hidden="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>IT-NAV-03</t>
+          <t>PT-FORM-02</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1162,7 +1114,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1185,14 +1137,14 @@
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>Harmonise, garde le nom le plus court</t>
+          <t>Joue ce test toi-même.</t>
         </is>
       </c>
     </row>
     <row r="18" hidden="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PT-CLICK-01</t>
+          <t>PT-HDR-01</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1223,16 +1175,12 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
+      <c r="J18" s="4" t="n"/>
     </row>
     <row r="19" hidden="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PT-HDR-01</t>
+          <t>PT-INPUT-01</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1263,7 +1211,11 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J19" s="4" t="n"/>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
     </row>
     <row r="20" hidden="1">
       <c r="A20" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Classeur de resultats final du 19/09 (session Tests de specifications)
Vue par defaut ramenee a 5 lignes : les 2 defauts mineurs restants (cle Web3Forms non restreinte,
DMARC absent) et les 3 points necessitant un acces dont l assistant ne dispose pas
(CAA et verrou registrar, reglages organisation GitHub, comportement de cache en production).
Aucun defaut de code ouvert.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_notes/validation/resultats-tests-site-web-20260919a.xlsx
+++ b/_notes/validation/resultats-tests-site-web-20260919a.xlsx
@@ -477,7 +477,7 @@
     <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Un seul onglet, 2 defauts (echecs) + 6 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
+          <t>Un seul onglet, 2 defauts (echecs) + 3 bloques + les points deja traites (trace conservee). Le classeur s'ouvre FILTRE sur l'ETAT REEL (colonne 'Gravite') : il montre ce qui attend encore quelque chose - les defauts ouverts et les cas encore bloques (y compris ceux qui attendent une action ou un accord de votre part, meme si vous avez deja ecrit 'Corriger') - et masque les points resolus ou deja executes. Une decision ecrite ne ferme pas un point tant qu'il n'est pas corrige. Pour revoir tout l'historique (points resolus / tests deja joues au navigateur), enlevez le filtre de la colonne 'Gravite'. Les defauts sont en haut, puis les cas bloques (Gravite='Bloque' : test non joue - la colonne 'Ce qui ne va pas' dit pourquoi), puis les points resolus. Remplissez 'Action souhaitee' (menu deroulant) ; cellules a remplir en jaune. Les cas en reussite ne sont pas listes.</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-03</t>
+          <t>PT-SUPPLY-01</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
@@ -703,22 +703,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Privacy of submissions</t>
+          <t>Supply chain</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -740,7 +740,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-04</t>
+          <t>ST-PERF-03</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -750,32 +750,32 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Bot / spam traps and key scraping</t>
+          <t>cache behaviour after a publication</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Envoi réel du formulaire de contact via le relais Web3Forms : nécessite ton accord (un vrai message part) et/ou l'accès au compte Web3Forms. À faire ensemble, pas en automatique.</t>
+          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Aucun défaut détecté : à vérifier avec un envoi de test contrôlé.</t>
+          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Envoi/relais Web3Forms de bout en bout (anti-spam, limitation d'envois) : demande l'accès au service et l'accord pour un envoi réel.</t>
+          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Toi (accès ou accord requis)</t>
+          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
@@ -789,99 +789,71 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-01</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>IT-FORM-02</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test d'intégration</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Supply chain</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Recherche de secrets et d'historique sensible dans le dépôt public du site : nécessite un outil dédié (gitleaks/trufflehog) et l'accès au dépôt.</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : audit à lancer sur le dépôt.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Scan de secrets / historique du dépôt public (gitleaks/trufflehog) et revue de la chaîne d'approvisionnement. Nécessite l'accès au dépôt.</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Toi (accès ou accord requis)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+      <c r="J10" s="4" t="n"/>
+    </row>
+    <row r="11" hidden="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>ST-CONTACT-02</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>IT-FORM-03</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intégration</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>same from EN</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -893,47 +865,35 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ST-PERF-03</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Bloqué</t>
+          <t>IT-NAV-03</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Résolu</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Test système (navigateur)</t>
+          <t>Test d'intégration</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>cache behaviour after a publication</t>
+          <t>(déjà traité lors d'un test précédent)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Test à faire à la main dans un navigateur (Chrome, Edge, Firefox, Safari iOS ; ordinateur et mobile) : c'est un parcours visuel de bout en bout. Il n'est pas rejoué automatiquement ici (le contrôle automatique lit le code des pages, pas leur rendu à l'écran). À réaliser par le testeur. Le détail du parcours est en colonne « Où ».</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Aucun défaut détecté : parcours à jouer manuellement pour confirmation.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Test système (ST) — scénario navigateur multi-appareils. Nécessite un vrai navigateur ; hors du périmètre du contrôle automatique du code source.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Testeur (navigateur : Chrome / Edge / Firefox / Safari iOS)</t>
-        </is>
-      </c>
+          <t>Ce point avait été signalé et vous aviez indiqué une action ; il n'apparaît plus dans les résultats (corrigé ou plus détecté). Ligne conservée pour la trace.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="4" t="inlineStr">
         <is>
           <t>Corriger</t>
@@ -941,14 +901,14 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Joue ce test toi-même.</t>
+          <t>Harmonise, garde le nom le plus court</t>
         </is>
       </c>
     </row>
     <row r="13" hidden="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>IT-FORM-02</t>
+          <t>PT-CLICK-01</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -958,7 +918,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -979,12 +939,16 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J13" s="4" t="n"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
     </row>
     <row r="14" hidden="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>IT-FORM-03</t>
+          <t>PT-FORM-02</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
@@ -994,7 +958,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1024,7 +988,7 @@
     <row r="15" hidden="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>IT-NAV-03</t>
+          <t>PT-FORM-03</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
@@ -1034,7 +998,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Test d'intégration</t>
+          <t>Test d'intrusion</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1057,14 +1021,14 @@
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>Harmonise, garde le nom le plus court</t>
+          <t>Joue ce test toi-même.</t>
         </is>
       </c>
     </row>
     <row r="16" hidden="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>PT-CLICK-01</t>
+          <t>PT-FORM-04</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
@@ -1104,7 +1068,7 @@
     <row r="17" hidden="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>PT-FORM-02</t>
+          <t>PT-HDR-01</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -1135,16 +1099,12 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>Joue ce test toi-même.</t>
-        </is>
-      </c>
+      <c r="J17" s="4" t="n"/>
     </row>
     <row r="18" hidden="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>PT-HDR-01</t>
+          <t>PT-INPUT-01</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
@@ -1175,12 +1135,16 @@
           <t>Corriger</t>
         </is>
       </c>
-      <c r="J18" s="4" t="n"/>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>Joue ce test toi-même.</t>
+        </is>
+      </c>
     </row>
     <row r="19" hidden="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>PT-INPUT-01</t>
+          <t>PT-PRIV-01</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
@@ -1220,7 +1184,7 @@
     <row r="20" hidden="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>PT-PRIV-01</t>
+          <t>PT-SUPPLY-02</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
@@ -1260,7 +1224,7 @@
     <row r="21" hidden="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>PT-SUPPLY-02</t>
+          <t>PT-TLS-02</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
@@ -1300,7 +1264,7 @@
     <row r="22" hidden="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PT-TLS-02</t>
+          <t>ST-A11Y-02</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -1310,7 +1274,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Test d'intrusion</t>
+          <t>Test système (navigateur)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1340,7 +1304,7 @@
     <row r="23" hidden="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-02</t>
+          <t>ST-A11Y-03</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -1380,7 +1344,7 @@
     <row r="24" hidden="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-03</t>
+          <t>ST-A11Y-04</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -1420,7 +1384,7 @@
     <row r="25" hidden="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-04</t>
+          <t>ST-A11Y-05</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
@@ -1460,7 +1424,7 @@
     <row r="26" hidden="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>ST-A11Y-05</t>
+          <t>ST-CONTACT-02</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">

</xml_diff>